<commit_message>
Clarify independent identity and demo floor-model provenance
</commit_message>
<xml_diff>
--- a/artifacts/exports/shuori-demo-events.xlsx
+++ b/artifacts/exports/shuori-demo-events.xlsx
@@ -47,7 +47,7 @@
     <t>守織 SHUORI · Workbook overview</t>
   </si>
   <si>
-    <t>Generated 2026-10-08 17:07:07 JST · Asia/Tokyo · demo · version 1.3.0</t>
+    <t>Generated 2026-10-08 17:31:56 JST · Asia/Tokyo · demo · version 1.3.0</t>
   </si>
   <si>
     <t>events | Exact selected IDs: 3 | View label: 3 matching events</t>
@@ -295,7 +295,7 @@
     <t>library</t>
   </si>
   <si>
-    <t>Nikoniko Bunko Plus</t>
+    <t>Library</t>
   </si>
   <si>
     <t>6F</t>
@@ -1406,10 +1406,10 @@
         <v>1</v>
       </c>
       <c r="K6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="L6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1442,10 +1442,10 @@
         <v>1</v>
       </c>
       <c r="K7" s="13">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="L7" s="13">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
   </sheetData>
@@ -1766,10 +1766,10 @@
         <v>1</v>
       </c>
       <c r="Y6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="Z6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
@@ -1840,10 +1840,10 @@
         <v>1</v>
       </c>
       <c r="Y7" s="13">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="Z7" s="13">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
@@ -1912,10 +1912,10 @@
         <v>1</v>
       </c>
       <c r="Y8" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="Z8" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
   </sheetData>
@@ -2914,10 +2914,10 @@
         <v>1</v>
       </c>
       <c r="N6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="O6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
   </sheetData>
@@ -3232,10 +3232,10 @@
         <v>1</v>
       </c>
       <c r="H6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="I6" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3261,10 +3261,10 @@
         <v>1</v>
       </c>
       <c r="H7" s="13">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="I7" s="13">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3290,10 +3290,10 @@
         <v>1</v>
       </c>
       <c r="H8" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
       <c r="I8" s="10">
-        <v>46303.70653649306</v>
+        <v>46303.72960831018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add printable PDF and Excel schedule and event views
</commit_message>
<xml_diff>
--- a/artifacts/exports/shuori-demo-events.xlsx
+++ b/artifacts/exports/shuori-demo-events.xlsx
@@ -47,7 +47,7 @@
     <t>守織 SHUORI · Workbook overview</t>
   </si>
   <si>
-    <t>Generated 2026-10-08 17:31:56 JST · Asia/Tokyo · demo · version 1.3.0</t>
+    <t>Generated 2026-10-08 18:03:49 JST · Asia/Tokyo · demo · version 1.4.0</t>
   </si>
   <si>
     <t>events | Exact selected IDs: 3 | View label: 3 matching events</t>
@@ -1406,10 +1406,10 @@
         <v>1</v>
       </c>
       <c r="K6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="L6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1442,10 +1442,10 @@
         <v>1</v>
       </c>
       <c r="K7" s="13">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="L7" s="13">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
   </sheetData>
@@ -1766,10 +1766,10 @@
         <v>1</v>
       </c>
       <c r="Y6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="Z6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
@@ -1840,10 +1840,10 @@
         <v>1</v>
       </c>
       <c r="Y7" s="13">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="Z7" s="13">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
@@ -1912,10 +1912,10 @@
         <v>1</v>
       </c>
       <c r="Y8" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="Z8" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
   </sheetData>
@@ -2914,10 +2914,10 @@
         <v>1</v>
       </c>
       <c r="N6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="O6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
   </sheetData>
@@ -3232,10 +3232,10 @@
         <v>1</v>
       </c>
       <c r="H6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="I6" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3261,10 +3261,10 @@
         <v>1</v>
       </c>
       <c r="H7" s="13">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="I7" s="13">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3290,10 +3290,10 @@
         <v>1</v>
       </c>
       <c r="H8" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
       <c r="I8" s="10">
-        <v>46303.72960831018</v>
+        <v>46303.745052638886</v>
       </c>
     </row>
   </sheetData>

</xml_diff>